<commit_message>
saucer handling for wiz modes, attract credits screen
</commit_message>
<xml_diff>
--- a/docs/final/spiderman_1967_50_villain_chapter_plan.xlsx
+++ b/docs/final/spiderman_1967_50_villain_chapter_plan.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc979030c4c5e40bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="Ra24d36874cbd4a3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R9131dd8c6ca9413d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="Ra7742a5233b34b30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R68b6253122b24608"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="Rb2eef1e1397f48ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Rce3c64ae7c2f46d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R51c3ffb6f2e14070"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Ra8ef8564b9444f1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Rb2068dd5bb2146d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R0c2e91afa1dc4a1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="Radf029c55689415d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="Rc91ff6af251846cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R42e6a8aaec184779"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R1866e8dd7e214faf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R06b05a59f8a540ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="Rc65d8e571aed4b48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="Ra12d42308d874097"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R7366b286c3de4010"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Ra1cc16b14bd04f4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Rfb124b67aaa647ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R1dc40669ff714c20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Rcbaff3af4c574db4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R6bdb444eef3c420f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R1fbd61e3790d4473"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R4d3ed572c8834407"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10054,7 +10054,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="120" customHeight="1">
       <x:c r="A2" s="31" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -10083,13 +10083,11 @@
           <x:t xml:space="preserve">No individual Case File powers. Each Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files; 0–500K). Ordinary switch, spinner, target, progress, and other non-jackpot scoring do not receive this bonus.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G2" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Approved/coded; needs machine playtest and polish.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="3">
+      <x:c r="G2" s="31" t="str">
+        <x:v>Coded; machine test pending. Up to 3 parked, 1 loose; 20s each. Goblin: release all on entry, 10s capture. Red pulse available; 75% red held; white flash objective. A+B adds below 4 balls.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="120" customHeight="1">
       <x:c r="A3" s="31" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -10118,13 +10116,11 @@
           <x:t xml:space="preserve">No individual Case File powers. Each Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files; 0–500K). Ordinary switch, spinner, target, progress, and other non-jackpot scoring do not receive this bonus.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G3" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Functional provisional implementation; design review and approval still required.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="4">
+      <x:c r="G3" s="31" t="str">
+        <x:v>Coded; machine test pending. Phase 1/Mysterio: up to 3 parked, 1 loose. Doc: none. Super: max 1. Independent 20s holds, oldest-ball recovery, staggered cleanup. White objective; red pulse available; 75% red held.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="120" customHeight="1">
       <x:c r="A4" s="31" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -10153,13 +10149,11 @@
           <x:t xml:space="preserve">No individual Case File powers. Each Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files; 0–500K). Ordinary switch, spinner, target, progress, and other non-jackpot scoring do not receive this bonus.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G4" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Approved/coded; needs machine playtest and polish.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="5">
+      <x:c r="G4" s="31" t="str">
+        <x:v>Coded; machine test pending. Up to 3 parked, 1 loose. Independent 12s holds. Cyclops releases one random ball. Oldest-ball recovery, duplicate-hit protection, staggered cleanup. White objective; red pulse available; 75% red held.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="120" customHeight="1">
       <x:c r="A5" s="31" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -10188,13 +10182,11 @@
           <x:t xml:space="preserve">No individual Case File powers. Each Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files; 0–500K). Ordinary switch, spinner, target, progress, and other non-jackpot scoring do not receive this bonus.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G5" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Functional provisional implementation; design review and approval still required.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="6">
+      <x:c r="G5" s="31" t="str">
+        <x:v>Coded; machine test pending. Up to 3 parked, 1 loose. Independent 15s holds. Drain checks and oldest-ball recovery. Matching rooftop award scores live 2x then releases that ball. Common lighting, duplicate protection and staggered cleanup.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="120" customHeight="1">
       <x:c r="A6" s="31" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -10223,13 +10215,11 @@
           <x:t xml:space="preserve">No individual Case File powers. Each Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files; 0–500K). Ordinary switch, spinner, target, progress, and other non-jackpot scoring do not receive this bonus.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G6" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Explicit placeholder shell; full design and coding required.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="7">
+      <x:c r="G6" s="31" t="str">
+        <x:v>Coded; machine test pending. VUK-aware parking. Independent 20s holds. Retain at most 1 between phases, timer continues. Oldest drain recovery, common lighting, staggered end release. Fiddler WATCH and 6s/2s Super releases preserved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="120" customHeight="1">
       <x:c r="A7" s="31" t="n">
         <x:v>6</x:v>
       </x:c>
@@ -10259,10 +10249,10 @@
         </x:is>
       </x:c>
       <x:c r="G7" s="31" t="str">
-        <x:v>Functional provisional implementation; design review and approval still required. Recent VUK timing fix: active gameplay VUK visits use the shared 1.5-second delayed release for both unlit and Curse Jackpot shots; the post-introduction launch remains immediate. Physical timing needs playtest.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
+        <x:v>Coded; machine test pending. Up to 3 parked, 1 loose. Independent 20s holds. Oldest drain recovery, common saucer lighting, staggered cleanup. Ruby scores then releases after 2s; pending releases cannot requalify or rescore.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="120" customHeight="1">
       <x:c r="A8" s="31" t="n">
         <x:v>7</x:v>
       </x:c>
@@ -10291,13 +10281,11 @@
           <x:t xml:space="preserve">No individual Case File powers. Each Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files; 0–500K). Ordinary switch, spinner, target, progress, and other non-jackpot scoring do not receive this bonus.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G8" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Explicit placeholder shell; full design and coding required.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="9">
+      <x:c r="G8" s="31" t="str">
+        <x:v>Coded; machine test pending. Up to 3 parked, 1 loose. Noah multiplier 1x–4x. Independent 20s holds. Oldest drain recovery, common saucer lighting. Noah scores before releasing all; 300ms staggering at collect and mode end.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="120" customHeight="1">
       <x:c r="A9" s="31" t="n">
         <x:v>8</x:v>
       </x:c>
@@ -10327,10 +10315,10 @@
         </x:is>
       </x:c>
       <x:c r="G9" s="31" t="str">
-        <x:v>Implemented repeating elemental-chain multiball; Blotto attack now accumulates up to three simultaneous solid-purple blocked zones during the thaw stage, with attack cadence 8s / 7s / 6s by cycle. Star clears all blocked zones and resets the timer. Needs machine playtest/polish.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
+        <x:v>Coded; machine test pending. Up to 3 parked, 1 loose. 20s holds; occupied hits remain active and refresh timers. Oldest drain recovery, common lighting, staggered end release. Qualifications persist through later stages. 5-ball cap retained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="120" customHeight="1">
       <x:c r="A10" s="31" t="n">
         <x:v>9</x:v>
       </x:c>
@@ -10360,10 +10348,10 @@
         </x:is>
       </x:c>
       <x:c r="G10" s="31" t="str">
-        <x:v>Implemented 3-ball VUK/saucer relay wizard cycling Igor, Molemen, and DeVargas lower phases into escalating Doctor Atlantean rooftop jackpots; needs machine playtest/polish.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
+        <x:v>Coded; machine test pending. VUK-aware parking, 20s holds. Oldest recovery on drain, VUK claim and continuous guard. Common lighting, 300ms end release, direct-stop VUK eject. Relay awards and occupied-hit protection retained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="120" customHeight="1">
       <x:c r="A11" s="31" t="n">
         <x:v>10</x:v>
       </x:c>
@@ -10392,13 +10380,11 @@
           <x:t xml:space="preserve">No individual Case File powers. Each Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files; 0–500K). Ordinary switch, spinner, target, progress, and other non-jackpot scoring do not receive this bonus.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G11" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Explicit placeholder shell; full design and coding required.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="12">
+      <x:c r="G11" s="31" t="str">
+        <x:v>Coded; machine test pending. 20s holds, up to 3 parked with 1 loose. Oldest drain recovery and 250ms guard. Common saucer lighting; 300ms multi-release spacing. Cameo/Brutus clearing and 500/750ms collection eject retained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="120" customHeight="1">
       <x:c r="A12" s="31" t="n">
         <x:v>11</x:v>
       </x:c>
@@ -10427,10 +10413,8 @@
           <x:t xml:space="preserve">No individual Case File powers. Each Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files; 0–500K). Ordinary switch, spinner, target, progress, and other non-jackpot scoring do not receive this bonus.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G12" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Explicit placeholder shell; full design and coding required.</x:t>
-        </x:is>
+      <x:c r="G12" s="31" t="str">
+        <x:v>Coded; machine test pending. 15s holds retained. Up to 3 parked with 1 loose; oldest drain recovery and 250ms guard. Common saucer lighting. Occupied reactivation hits can collect objectives; original timers/order retained. Timers persist across phases; 300ms end release.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">

</xml_diff>